<commit_message>
Fix Excel template filename
</commit_message>
<xml_diff>
--- a/dist/HRVec-Andaman2-Personnel-Template.xlsx
+++ b/dist/HRVec-Andaman2-Personnel-Template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="บุคลากร" sheetId="1" r:id="Rc7c057a5df8f4a6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ใบรับรองวิชาชีพ" sheetId="2" r:id="Ra4f4f8df49bc48ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="คำแนะนำ" sheetId="3" r:id="R3e322442249249e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="รายการอ้างอิง" sheetId="4" r:id="Rd70ef3d98b5a4a45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่าง" sheetId="5" r:id="Rb2ba1f3992a14f90"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่างใบรับรอง" sheetId="6" r:id="R0ba9a666ff4943dc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="บุคลากร" sheetId="1" r:id="R4bae220c9bbf4798"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ใบรับรองวิชาชีพ" sheetId="2" r:id="R5a41ef67af4a40b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="คำแนะนำ" sheetId="3" r:id="R5ca24f1a556a40d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="รายการอ้างอิง" sheetId="4" r:id="R882bce3f9a1f4c61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่าง" sheetId="5" r:id="Racd4f71885eb48e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่างใบรับรอง" sheetId="6" r:id="Rc16419410df7443c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8854,25 +8854,25 @@
     <x:dataValidation type="list" sqref="B2:B501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$I$2:$I$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$I$2:$I$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="C2:C501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="C2:C501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$J$2:$J$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$J$2:$J$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="D2:D501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="D2:D501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$K$2:$K$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$K$2:$K$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="E2:E501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="E2:E501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!"&amp;IF(IFERROR(VLOOKUP($C2,'รายการอ้างอิง'!$B$2:$D$9,3,0),"")="ส่วนกลางสถาบัน","AC2:AC1001","AB2:AB1001"))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$M$2:$M$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$M$2:$M$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="G2:G501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="G2:G501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$N$2:$N$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$N$2:$N$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="กรอกวันที่ วว/ดด/ปี พ.ศ." sqref="H2:H501">
+    <x:dataValidation type="custom" sqref="H2:H501">
       <x:formula1>OR(H2="",ISNUMBER(H2),AND(ISTEXT(H2),LEN(H2)&gt;=8,LEN(H2)&lt;=10))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="กรอกวันที่ วว/ดด/ปี พ.ศ." sqref="I2:I501">
+    <x:dataValidation type="custom" sqref="I2:I501">
       <x:formula1>OR(I2="",ISNUMBER(I2),AND(ISTEXT(I2),LEN(I2)&gt;=8,LEN(I2)&lt;=10))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J2:J501">
@@ -8887,7 +8887,7 @@
     <x:dataValidation type="list" sqref="M2:M501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$R$2:$R$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$R$2:$R$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="N2:N501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="N2:N501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$S$2:$S$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$S$2:$S$1001)+1))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="O2:O501">
@@ -68948,10 +68948,10 @@
     </x:row>
   </x:sheetData>
   <x:dataValidations count="10">
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="A2:A5001">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="A2:A5001">
       <x:formula1>INDIRECT("'บุคลากร'!$A$2:$A$"&amp;MAX(2,COUNTA('บุคลากร'!$A$2:$A$501)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="B2:B5001">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="B2:B5001">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$U$2:$U$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$U$2:$U$1001)+1))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C5001">
@@ -68963,10 +68963,10 @@
     <x:dataValidation type="list" sqref="E2:E5001">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$X$2:$X$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$X$2:$X$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="กรอกวันที่ วว/ดด/ปี พ.ศ." sqref="F2:F5001">
+    <x:dataValidation type="custom" sqref="F2:F5001">
       <x:formula1>OR(F2="",ISNUMBER(F2),AND(ISTEXT(F2),LEN(F2)&gt;=8,LEN(F2)&lt;=10))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="กรอกวันที่ วว/ดด/ปี พ.ศ." sqref="G2:G5001">
+    <x:dataValidation type="custom" sqref="G2:G5001">
       <x:formula1>OR(G2="",ISNUMBER(G2),AND(ISTEXT(G2),LEN(G2)&gt;=8,LEN(G2)&lt;=10))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="H2:H5001">
@@ -69004,7 +69004,7 @@
         <x:v>รุ่นแม่แบบ</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>HRVec-Andaman2 รุ่น 1.12 รายการเลือกตรงกับฟอร์ม</x:v>
+        <x:v>HRVec-Andaman2 รุ่น 1.10 วันที่ พ.ศ. และรายการเลือก</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -69060,7 +69060,7 @@
         <x:v>รายการเลือก</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>เลือกเซลล์แล้วกดลูกศรด้านขวาหรือ Alt + ลูกศรลง หน่วยงาน ตำแหน่ง ฝ่าย วิทยฐานะ วุฒิ ตำแหน่งทางวิชาการ ด้านงาน และประเภทใบรับรองอ้างอิงรายการเดียวกับฟอร์ม</x:v>
+        <x:v>กดเซลล์แล้วเลือกลูกศร ช่องข้อความเพิ่มเติมกรอกเองได้ รายการอ้างอิงตั้งแต่คอลัมน์ H แก้หรือเพิ่มต่อเนื่องได้ถึงแถว 1001</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -69144,12 +69144,7 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
-      <x:c r="A20" s="1" t="str">
-        <x:v>รายการล่าสุด</x:v>
-      </x:c>
-      <x:c r="B20" s="7" t="str">
-        <x:v>เมื่อแอดมินเพิ่มรายการในระบบ ให้ดาวน์โหลดแม่แบบจากเว็บใหม่ ไฟล์ Excel ที่บันทึกไว้แล้วไม่เปลี่ยนตามระบบอัตโนมัติ</x:v>
-      </x:c>
+      <x:c r="B20" s="8"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -69274,7 +69269,7 @@
         <x:v>ส่วนราชการสถาบัน</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="15" hidden="0" customHeight="1">
+    <x:row r="2">
       <x:c r="A2" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -69298,7 +69293,7 @@
       <x:c r="K2" s="1" t="str">
         <x:v>ครู</x:v>
       </x:c>
-      <x:c r="L2" s="7" t="str">
+      <x:c r="L2" s="1" t="str">
         <x:v>ฝ่ายบริหารทรัพยากร</x:v>
       </x:c>
       <x:c r="M2" s="1"/>
@@ -69315,7 +69310,7 @@
         <x:v>อาจารย์</x:v>
       </x:c>
       <x:c r="T2" s="1" t="str">
-        <x:v>การเงินและบัญชี</x:v>
+        <x:v>บริหารงานบุคคล</x:v>
       </x:c>
       <x:c r="U2" s="1" t="str">
         <x:v>ใบประกอบวิชาชีพผู้บริหาร</x:v>
@@ -69333,7 +69328,7 @@
         <x:v>สำนักงานผู้อำนวยการสถาบัน</x:v>
       </x:c>
     </x:row>
-    <x:row r="3" ht="15" hidden="0" customHeight="1">
+    <x:row r="3">
       <x:c r="A3" s="1" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -69357,7 +69352,7 @@
       <x:c r="K3" s="1" t="str">
         <x:v>ครูผู้ช่วย</x:v>
       </x:c>
-      <x:c r="L3" s="7" t="str">
+      <x:c r="L3" s="1" t="str">
         <x:v>ฝ่ายยุทธศาสตร์และแผนงาน</x:v>
       </x:c>
       <x:c r="M3" s="1"/>
@@ -69374,7 +69369,7 @@
         <x:v>ผู้ช่วยศาสตราจารย์</x:v>
       </x:c>
       <x:c r="T3" s="1" t="str">
-        <x:v>เทคโนโลยีสารสนเทศ</x:v>
+        <x:v>การเงินและบัญชี</x:v>
       </x:c>
       <x:c r="U3" s="1" t="str">
         <x:v>ใบรับรองทักษะวิชาชีพ</x:v>
@@ -69392,7 +69387,7 @@
         <x:v>สำนักพัฒนายุทธศาสตร์และความร่วมมืออาชีวศึกษา</x:v>
       </x:c>
     </x:row>
-    <x:row r="4" ht="15" hidden="0" customHeight="1">
+    <x:row r="4">
       <x:c r="A4" s="1" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -69416,7 +69411,7 @@
       <x:c r="K4" s="1" t="str">
         <x:v>เจ้าหน้าที่</x:v>
       </x:c>
-      <x:c r="L4" s="7" t="str">
+      <x:c r="L4" s="1" t="str">
         <x:v>ฝ่ายกิจการนักเรียน นักศึกษา</x:v>
       </x:c>
       <x:c r="M4" s="1"/>
@@ -69433,7 +69428,7 @@
         <x:v>รองศาสตราจารย์</x:v>
       </x:c>
       <x:c r="T4" s="1" t="str">
-        <x:v>บริหารงานบุคคล</x:v>
+        <x:v>พัสดุ</x:v>
       </x:c>
       <x:c r="U4" s="1" t="str">
         <x:v>ใบรับรองสมรรถนะทางวิชาชีพ</x:v>
@@ -69451,7 +69446,7 @@
         <x:v>สำนักพัฒนากิจการนักศึกษาและกิจการพิเศษ</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="15" hidden="0" customHeight="1">
+    <x:row r="5">
       <x:c r="A5" s="1" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -69475,7 +69470,7 @@
       <x:c r="K5" s="1" t="str">
         <x:v>ผู้ช่วยผู้อำนวยการสถาบัน</x:v>
       </x:c>
-      <x:c r="L5" s="7" t="str">
+      <x:c r="L5" s="1" t="str">
         <x:v>ฝ่ายวิชาการ</x:v>
       </x:c>
       <x:c r="M5" s="1"/>
@@ -69492,7 +69487,7 @@
         <x:v>ศาสตราจารย์</x:v>
       </x:c>
       <x:c r="T5" s="1" t="str">
-        <x:v>ประสานงานและความร่วมมือ</x:v>
+        <x:v>แผนงานและงบประมาณ</x:v>
       </x:c>
       <x:c r="U5" s="1" t="str">
         <x:v>ใบประกอบวิชาชีพครู</x:v>
@@ -69510,7 +69505,7 @@
         <x:v>ศูนย์วิจัยและพัฒนาการอาชีวศึกษา</x:v>
       </x:c>
     </x:row>
-    <x:row r="6" ht="15" hidden="0" customHeight="1">
+    <x:row r="6">
       <x:c r="A6" s="1" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -69534,7 +69529,7 @@
       <x:c r="K6" s="1" t="str">
         <x:v>ผู้อำนวยการ</x:v>
       </x:c>
-      <x:c r="L6" s="7" t="str">
+      <x:c r="L6" s="1" t="str">
         <x:v>สำนักงานผู้อำนวยการสถาบัน</x:v>
       </x:c>
       <x:c r="M6" s="1"/>
@@ -69549,7 +69544,7 @@
       <x:c r="R6" s="1"/>
       <x:c r="S6" s="1"/>
       <x:c r="T6" s="1" t="str">
-        <x:v>แผนงานและงบประมาณ</x:v>
+        <x:v>เทคโนโลยีสารสนเทศ</x:v>
       </x:c>
       <x:c r="U6" s="1"/>
       <x:c r="V6" s="1"/>
@@ -69563,7 +69558,7 @@
         <x:v>อาชีวศึกษาบัณฑิต</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
+    <x:row r="7">
       <x:c r="A7" s="1" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -69587,7 +69582,7 @@
       <x:c r="K7" s="1" t="str">
         <x:v>ผู้อำนวยการศูนย์</x:v>
       </x:c>
-      <x:c r="L7" s="7" t="str">
+      <x:c r="L7" s="1" t="str">
         <x:v>สำนักพัฒนายุทธศาสตร์และความร่วมมืออาชีวศึกษา</x:v>
       </x:c>
       <x:c r="M7" s="1"/>
@@ -69600,7 +69595,7 @@
       <x:c r="R7" s="1"/>
       <x:c r="S7" s="1"/>
       <x:c r="T7" s="1" t="str">
-        <x:v>พัสดุ</x:v>
+        <x:v>สารบรรณและธุรการ</x:v>
       </x:c>
       <x:c r="U7" s="1"/>
       <x:c r="V7" s="1"/>
@@ -69612,7 +69607,7 @@
       <x:c r="AB7" s="1"/>
       <x:c r="AC7" s="1"/>
     </x:row>
-    <x:row r="8" ht="15" hidden="0" customHeight="1">
+    <x:row r="8">
       <x:c r="A8" s="1" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -69636,7 +69631,7 @@
       <x:c r="K8" s="1" t="str">
         <x:v>ผู้อำนวยการสถาบัน</x:v>
       </x:c>
-      <x:c r="L8" s="7" t="str">
+      <x:c r="L8" s="1" t="str">
         <x:v>สำนักพัฒนากิจการนักศึกษาและกิจการพิเศษ</x:v>
       </x:c>
       <x:c r="M8" s="1"/>
@@ -69649,7 +69644,7 @@
       <x:c r="R8" s="1"/>
       <x:c r="S8" s="1"/>
       <x:c r="T8" s="1" t="str">
-        <x:v>สารบรรณและธุรการ</x:v>
+        <x:v>ประสานงานและความร่วมมือ</x:v>
       </x:c>
       <x:c r="U8" s="1"/>
       <x:c r="V8" s="1"/>
@@ -69661,7 +69656,7 @@
       <x:c r="AB8" s="1"/>
       <x:c r="AC8" s="1"/>
     </x:row>
-    <x:row r="9" ht="15" hidden="0" customHeight="1">
+    <x:row r="9">
       <x:c r="A9" s="1" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -69685,7 +69680,7 @@
       <x:c r="K9" s="1" t="str">
         <x:v>ผู้อำนวยการสำนัก</x:v>
       </x:c>
-      <x:c r="L9" s="7" t="str">
+      <x:c r="L9" s="1" t="str">
         <x:v>ศูนย์วิจัยและพัฒนาการอาชีวศึกษา</x:v>
       </x:c>
       <x:c r="M9" s="1"/>
@@ -69708,7 +69703,7 @@
       <x:c r="AB9" s="1"/>
       <x:c r="AC9" s="1"/>
     </x:row>
-    <x:row r="10" ht="15" hidden="0" customHeight="1">
+    <x:row r="10">
       <x:c r="A10" s="1"/>
       <x:c r="B10" s="1"/>
       <x:c r="C10" s="1"/>
@@ -69722,7 +69717,7 @@
       <x:c r="K10" s="1" t="str">
         <x:v>ผู้อำนวยการสำนักงาน</x:v>
       </x:c>
-      <x:c r="L10" s="7" t="str">
+      <x:c r="L10" s="1" t="str">
         <x:v>อาชีวศึกษาบัณฑิต</x:v>
       </x:c>
       <x:c r="M10" s="1"/>
@@ -69761,7 +69756,7 @@
       <x:c r="I11" s="1"/>
       <x:c r="J11" s="1"/>
       <x:c r="K11" s="1" t="str">
-        <x:v>พนักงานบริหารงานทั่วไป</x:v>
+        <x:v>พนักงานราชการ</x:v>
       </x:c>
       <x:c r="L11" s="1"/>
       <x:c r="M11" s="1"/>
@@ -69800,7 +69795,7 @@
       <x:c r="I12" s="1"/>
       <x:c r="J12" s="1"/>
       <x:c r="K12" s="1" t="str">
-        <x:v>พนักงานราชการ</x:v>
+        <x:v>รองผู้อำนวยการ</x:v>
       </x:c>
       <x:c r="L12" s="1"/>
       <x:c r="M12" s="1"/>
@@ -69837,7 +69832,7 @@
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="1"/>
       <x:c r="K13" s="1" t="str">
-        <x:v>รองผู้อำนวยการ</x:v>
+        <x:v>รองผู้อำนวยการสถาบัน</x:v>
       </x:c>
       <x:c r="L13" s="1"/>
       <x:c r="M13" s="1"/>
@@ -69874,7 +69869,7 @@
       <x:c r="I14" s="1"/>
       <x:c r="J14" s="1"/>
       <x:c r="K14" s="1" t="str">
-        <x:v>รองผู้อำนวยการสถาบัน</x:v>
+        <x:v>หัวหน้างาน</x:v>
       </x:c>
       <x:c r="L14" s="1"/>
       <x:c r="M14" s="1"/>
@@ -69911,7 +69906,7 @@
       <x:c r="I15" s="1"/>
       <x:c r="J15" s="1"/>
       <x:c r="K15" s="1" t="str">
-        <x:v>หัวหน้างาน</x:v>
+        <x:v>อาจารย์</x:v>
       </x:c>
       <x:c r="L15" s="1"/>
       <x:c r="M15" s="1"/>
@@ -69948,7 +69943,7 @@
       <x:c r="I16" s="1"/>
       <x:c r="J16" s="1"/>
       <x:c r="K16" s="1" t="str">
-        <x:v>อาจารย์</x:v>
+        <x:v>พนักงานบริหารงานทั่วไป</x:v>
       </x:c>
       <x:c r="L16" s="1"/>
       <x:c r="M16" s="1"/>

</xml_diff>

<commit_message>
Sync all v1.12 template files
</commit_message>
<xml_diff>
--- a/dist/HRVec-Andaman2-Personnel-Template.xlsx
+++ b/dist/HRVec-Andaman2-Personnel-Template.xlsx
@@ -2,12 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="บุคลากร" sheetId="1" r:id="R4bae220c9bbf4798"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ใบรับรองวิชาชีพ" sheetId="2" r:id="R5a41ef67af4a40b6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="คำแนะนำ" sheetId="3" r:id="R5ca24f1a556a40d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="รายการอ้างอิง" sheetId="4" r:id="R882bce3f9a1f4c61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่าง" sheetId="5" r:id="Racd4f71885eb48e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่างใบรับรอง" sheetId="6" r:id="Rc16419410df7443c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="บุคลากร" sheetId="1" r:id="Rc7c057a5df8f4a6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ใบรับรองวิชาชีพ" sheetId="2" r:id="Ra4f4f8df49bc48ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="คำแนะนำ" sheetId="3" r:id="R3e322442249249e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="รายการอ้างอิง" sheetId="4" r:id="Rd70ef3d98b5a4a45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่าง" sheetId="5" r:id="Rb2ba1f3992a14f90"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ตัวอย่างใบรับรอง" sheetId="6" r:id="R0ba9a666ff4943dc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8854,25 +8854,25 @@
     <x:dataValidation type="list" sqref="B2:B501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$I$2:$I$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$I$2:$I$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="C2:C501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="C2:C501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$J$2:$J$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$J$2:$J$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="D2:D501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="D2:D501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$K$2:$K$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$K$2:$K$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="E2:E501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="E2:E501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!"&amp;IF(IFERROR(VLOOKUP($C2,'รายการอ้างอิง'!$B$2:$D$9,3,0),"")="ส่วนกลางสถาบัน","AC2:AC1001","AB2:AB1001"))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="F2:F501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$M$2:$M$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$M$2:$M$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="G2:G501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="G2:G501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$N$2:$N$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$N$2:$N$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" sqref="H2:H501">
+    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="กรอกวันที่ วว/ดด/ปี พ.ศ." sqref="H2:H501">
       <x:formula1>OR(H2="",ISNUMBER(H2),AND(ISTEXT(H2),LEN(H2)&gt;=8,LEN(H2)&lt;=10))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" sqref="I2:I501">
+    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="กรอกวันที่ วว/ดด/ปี พ.ศ." sqref="I2:I501">
       <x:formula1>OR(I2="",ISNUMBER(I2),AND(ISTEXT(I2),LEN(I2)&gt;=8,LEN(I2)&lt;=10))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="J2:J501">
@@ -8887,7 +8887,7 @@
     <x:dataValidation type="list" sqref="M2:M501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$R$2:$R$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$R$2:$R$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="N2:N501">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="N2:N501">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$S$2:$S$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$S$2:$S$1001)+1))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="O2:O501">
@@ -68948,10 +68948,10 @@
     </x:row>
   </x:sheetData>
   <x:dataValidations count="10">
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="A2:A5001">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="A2:A5001">
       <x:formula1>INDIRECT("'บุคลากร'!$A$2:$A$"&amp;MAX(2,COUNTA('บุคลากร'!$A$2:$A$501)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรายการ" error="กรุณาเลือกรายการจากข้อมูลอ้างอิง" sqref="B2:B5001">
+    <x:dataValidation type="list" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="เลือกรายการเดียวกับฟอร์มในระบบ" sqref="B2:B5001">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$U$2:$U$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$U$2:$U$1001)+1))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="C2:C5001">
@@ -68963,10 +68963,10 @@
     <x:dataValidation type="list" sqref="E2:E5001">
       <x:formula1>INDIRECT("'รายการอ้างอิง'!$X$2:$X$"&amp;MAX(2,COUNTA('รายการอ้างอิง'!$X$2:$X$1001)+1))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" sqref="F2:F5001">
+    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="กรอกวันที่ วว/ดด/ปี พ.ศ." sqref="F2:F5001">
       <x:formula1>OR(F2="",ISNUMBER(F2),AND(ISTEXT(F2),LEN(F2)&gt;=8,LEN(F2)&lt;=10))</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="custom" sqref="G2:G5001">
+    <x:dataValidation type="custom" errorStyle="stop" showErrorMessage="1" errorTitle="ข้อมูลไม่ตรงรูปแบบ" error="กรอกวันที่ วว/ดด/ปี พ.ศ." sqref="G2:G5001">
       <x:formula1>OR(G2="",ISNUMBER(G2),AND(ISTEXT(G2),LEN(G2)&gt;=8,LEN(G2)&lt;=10))</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="H2:H5001">
@@ -69004,7 +69004,7 @@
         <x:v>รุ่นแม่แบบ</x:v>
       </x:c>
       <x:c r="B2" s="7" t="str">
-        <x:v>HRVec-Andaman2 รุ่น 1.10 วันที่ พ.ศ. และรายการเลือก</x:v>
+        <x:v>HRVec-Andaman2 รุ่น 1.12 รายการเลือกตรงกับฟอร์ม</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="48" customHeight="1">
@@ -69060,7 +69060,7 @@
         <x:v>รายการเลือก</x:v>
       </x:c>
       <x:c r="B9" s="7" t="str">
-        <x:v>กดเซลล์แล้วเลือกลูกศร ช่องข้อความเพิ่มเติมกรอกเองได้ รายการอ้างอิงตั้งแต่คอลัมน์ H แก้หรือเพิ่มต่อเนื่องได้ถึงแถว 1001</x:v>
+        <x:v>เลือกเซลล์แล้วกดลูกศรด้านขวาหรือ Alt + ลูกศรลง หน่วยงาน ตำแหน่ง ฝ่าย วิทยฐานะ วุฒิ ตำแหน่งทางวิชาการ ด้านงาน และประเภทใบรับรองอ้างอิงรายการเดียวกับฟอร์ม</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="48" customHeight="1">
@@ -69144,7 +69144,12 @@
       </x:c>
     </x:row>
     <x:row r="20" ht="48" customHeight="1">
-      <x:c r="B20" s="8"/>
+      <x:c r="A20" s="1" t="str">
+        <x:v>รายการล่าสุด</x:v>
+      </x:c>
+      <x:c r="B20" s="7" t="str">
+        <x:v>เมื่อแอดมินเพิ่มรายการในระบบ ให้ดาวน์โหลดแม่แบบจากเว็บใหม่ ไฟล์ Excel ที่บันทึกไว้แล้วไม่เปลี่ยนตามระบบอัตโนมัติ</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -69269,7 +69274,7 @@
         <x:v>ส่วนราชการสถาบัน</x:v>
       </x:c>
     </x:row>
-    <x:row r="2">
+    <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="1" t="n">
         <x:v>1</x:v>
       </x:c>
@@ -69293,7 +69298,7 @@
       <x:c r="K2" s="1" t="str">
         <x:v>ครู</x:v>
       </x:c>
-      <x:c r="L2" s="1" t="str">
+      <x:c r="L2" s="7" t="str">
         <x:v>ฝ่ายบริหารทรัพยากร</x:v>
       </x:c>
       <x:c r="M2" s="1"/>
@@ -69310,7 +69315,7 @@
         <x:v>อาจารย์</x:v>
       </x:c>
       <x:c r="T2" s="1" t="str">
-        <x:v>บริหารงานบุคคล</x:v>
+        <x:v>การเงินและบัญชี</x:v>
       </x:c>
       <x:c r="U2" s="1" t="str">
         <x:v>ใบประกอบวิชาชีพผู้บริหาร</x:v>
@@ -69328,7 +69333,7 @@
         <x:v>สำนักงานผู้อำนวยการสถาบัน</x:v>
       </x:c>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="1" t="n">
         <x:v>2</x:v>
       </x:c>
@@ -69352,7 +69357,7 @@
       <x:c r="K3" s="1" t="str">
         <x:v>ครูผู้ช่วย</x:v>
       </x:c>
-      <x:c r="L3" s="1" t="str">
+      <x:c r="L3" s="7" t="str">
         <x:v>ฝ่ายยุทธศาสตร์และแผนงาน</x:v>
       </x:c>
       <x:c r="M3" s="1"/>
@@ -69369,7 +69374,7 @@
         <x:v>ผู้ช่วยศาสตราจารย์</x:v>
       </x:c>
       <x:c r="T3" s="1" t="str">
-        <x:v>การเงินและบัญชี</x:v>
+        <x:v>เทคโนโลยีสารสนเทศ</x:v>
       </x:c>
       <x:c r="U3" s="1" t="str">
         <x:v>ใบรับรองทักษะวิชาชีพ</x:v>
@@ -69387,7 +69392,7 @@
         <x:v>สำนักพัฒนายุทธศาสตร์และความร่วมมืออาชีวศึกษา</x:v>
       </x:c>
     </x:row>
-    <x:row r="4">
+    <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="1" t="n">
         <x:v>3</x:v>
       </x:c>
@@ -69411,7 +69416,7 @@
       <x:c r="K4" s="1" t="str">
         <x:v>เจ้าหน้าที่</x:v>
       </x:c>
-      <x:c r="L4" s="1" t="str">
+      <x:c r="L4" s="7" t="str">
         <x:v>ฝ่ายกิจการนักเรียน นักศึกษา</x:v>
       </x:c>
       <x:c r="M4" s="1"/>
@@ -69428,7 +69433,7 @@
         <x:v>รองศาสตราจารย์</x:v>
       </x:c>
       <x:c r="T4" s="1" t="str">
-        <x:v>พัสดุ</x:v>
+        <x:v>บริหารงานบุคคล</x:v>
       </x:c>
       <x:c r="U4" s="1" t="str">
         <x:v>ใบรับรองสมรรถนะทางวิชาชีพ</x:v>
@@ -69446,7 +69451,7 @@
         <x:v>สำนักพัฒนากิจการนักศึกษาและกิจการพิเศษ</x:v>
       </x:c>
     </x:row>
-    <x:row r="5">
+    <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="1" t="n">
         <x:v>4</x:v>
       </x:c>
@@ -69470,7 +69475,7 @@
       <x:c r="K5" s="1" t="str">
         <x:v>ผู้ช่วยผู้อำนวยการสถาบัน</x:v>
       </x:c>
-      <x:c r="L5" s="1" t="str">
+      <x:c r="L5" s="7" t="str">
         <x:v>ฝ่ายวิชาการ</x:v>
       </x:c>
       <x:c r="M5" s="1"/>
@@ -69487,7 +69492,7 @@
         <x:v>ศาสตราจารย์</x:v>
       </x:c>
       <x:c r="T5" s="1" t="str">
-        <x:v>แผนงานและงบประมาณ</x:v>
+        <x:v>ประสานงานและความร่วมมือ</x:v>
       </x:c>
       <x:c r="U5" s="1" t="str">
         <x:v>ใบประกอบวิชาชีพครู</x:v>
@@ -69505,7 +69510,7 @@
         <x:v>ศูนย์วิจัยและพัฒนาการอาชีวศึกษา</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
+    <x:row r="6" ht="15" hidden="0" customHeight="1">
       <x:c r="A6" s="1" t="n">
         <x:v>5</x:v>
       </x:c>
@@ -69529,7 +69534,7 @@
       <x:c r="K6" s="1" t="str">
         <x:v>ผู้อำนวยการ</x:v>
       </x:c>
-      <x:c r="L6" s="1" t="str">
+      <x:c r="L6" s="7" t="str">
         <x:v>สำนักงานผู้อำนวยการสถาบัน</x:v>
       </x:c>
       <x:c r="M6" s="1"/>
@@ -69544,7 +69549,7 @@
       <x:c r="R6" s="1"/>
       <x:c r="S6" s="1"/>
       <x:c r="T6" s="1" t="str">
-        <x:v>เทคโนโลยีสารสนเทศ</x:v>
+        <x:v>แผนงานและงบประมาณ</x:v>
       </x:c>
       <x:c r="U6" s="1"/>
       <x:c r="V6" s="1"/>
@@ -69558,7 +69563,7 @@
         <x:v>อาชีวศึกษาบัณฑิต</x:v>
       </x:c>
     </x:row>
-    <x:row r="7">
+    <x:row r="7" ht="26.399999618530273" hidden="0" customHeight="1">
       <x:c r="A7" s="1" t="n">
         <x:v>6</x:v>
       </x:c>
@@ -69582,7 +69587,7 @@
       <x:c r="K7" s="1" t="str">
         <x:v>ผู้อำนวยการศูนย์</x:v>
       </x:c>
-      <x:c r="L7" s="1" t="str">
+      <x:c r="L7" s="7" t="str">
         <x:v>สำนักพัฒนายุทธศาสตร์และความร่วมมืออาชีวศึกษา</x:v>
       </x:c>
       <x:c r="M7" s="1"/>
@@ -69595,7 +69600,7 @@
       <x:c r="R7" s="1"/>
       <x:c r="S7" s="1"/>
       <x:c r="T7" s="1" t="str">
-        <x:v>สารบรรณและธุรการ</x:v>
+        <x:v>พัสดุ</x:v>
       </x:c>
       <x:c r="U7" s="1"/>
       <x:c r="V7" s="1"/>
@@ -69607,7 +69612,7 @@
       <x:c r="AB7" s="1"/>
       <x:c r="AC7" s="1"/>
     </x:row>
-    <x:row r="8">
+    <x:row r="8" ht="15" hidden="0" customHeight="1">
       <x:c r="A8" s="1" t="n">
         <x:v>7</x:v>
       </x:c>
@@ -69631,7 +69636,7 @@
       <x:c r="K8" s="1" t="str">
         <x:v>ผู้อำนวยการสถาบัน</x:v>
       </x:c>
-      <x:c r="L8" s="1" t="str">
+      <x:c r="L8" s="7" t="str">
         <x:v>สำนักพัฒนากิจการนักศึกษาและกิจการพิเศษ</x:v>
       </x:c>
       <x:c r="M8" s="1"/>
@@ -69644,7 +69649,7 @@
       <x:c r="R8" s="1"/>
       <x:c r="S8" s="1"/>
       <x:c r="T8" s="1" t="str">
-        <x:v>ประสานงานและความร่วมมือ</x:v>
+        <x:v>สารบรรณและธุรการ</x:v>
       </x:c>
       <x:c r="U8" s="1"/>
       <x:c r="V8" s="1"/>
@@ -69656,7 +69661,7 @@
       <x:c r="AB8" s="1"/>
       <x:c r="AC8" s="1"/>
     </x:row>
-    <x:row r="9">
+    <x:row r="9" ht="15" hidden="0" customHeight="1">
       <x:c r="A9" s="1" t="n">
         <x:v>8</x:v>
       </x:c>
@@ -69680,7 +69685,7 @@
       <x:c r="K9" s="1" t="str">
         <x:v>ผู้อำนวยการสำนัก</x:v>
       </x:c>
-      <x:c r="L9" s="1" t="str">
+      <x:c r="L9" s="7" t="str">
         <x:v>ศูนย์วิจัยและพัฒนาการอาชีวศึกษา</x:v>
       </x:c>
       <x:c r="M9" s="1"/>
@@ -69703,7 +69708,7 @@
       <x:c r="AB9" s="1"/>
       <x:c r="AC9" s="1"/>
     </x:row>
-    <x:row r="10">
+    <x:row r="10" ht="15" hidden="0" customHeight="1">
       <x:c r="A10" s="1"/>
       <x:c r="B10" s="1"/>
       <x:c r="C10" s="1"/>
@@ -69717,7 +69722,7 @@
       <x:c r="K10" s="1" t="str">
         <x:v>ผู้อำนวยการสำนักงาน</x:v>
       </x:c>
-      <x:c r="L10" s="1" t="str">
+      <x:c r="L10" s="7" t="str">
         <x:v>อาชีวศึกษาบัณฑิต</x:v>
       </x:c>
       <x:c r="M10" s="1"/>
@@ -69756,7 +69761,7 @@
       <x:c r="I11" s="1"/>
       <x:c r="J11" s="1"/>
       <x:c r="K11" s="1" t="str">
-        <x:v>พนักงานราชการ</x:v>
+        <x:v>พนักงานบริหารงานทั่วไป</x:v>
       </x:c>
       <x:c r="L11" s="1"/>
       <x:c r="M11" s="1"/>
@@ -69795,7 +69800,7 @@
       <x:c r="I12" s="1"/>
       <x:c r="J12" s="1"/>
       <x:c r="K12" s="1" t="str">
-        <x:v>รองผู้อำนวยการ</x:v>
+        <x:v>พนักงานราชการ</x:v>
       </x:c>
       <x:c r="L12" s="1"/>
       <x:c r="M12" s="1"/>
@@ -69832,7 +69837,7 @@
       <x:c r="I13" s="1"/>
       <x:c r="J13" s="1"/>
       <x:c r="K13" s="1" t="str">
-        <x:v>รองผู้อำนวยการสถาบัน</x:v>
+        <x:v>รองผู้อำนวยการ</x:v>
       </x:c>
       <x:c r="L13" s="1"/>
       <x:c r="M13" s="1"/>
@@ -69869,7 +69874,7 @@
       <x:c r="I14" s="1"/>
       <x:c r="J14" s="1"/>
       <x:c r="K14" s="1" t="str">
-        <x:v>หัวหน้างาน</x:v>
+        <x:v>รองผู้อำนวยการสถาบัน</x:v>
       </x:c>
       <x:c r="L14" s="1"/>
       <x:c r="M14" s="1"/>
@@ -69906,7 +69911,7 @@
       <x:c r="I15" s="1"/>
       <x:c r="J15" s="1"/>
       <x:c r="K15" s="1" t="str">
-        <x:v>อาจารย์</x:v>
+        <x:v>หัวหน้างาน</x:v>
       </x:c>
       <x:c r="L15" s="1"/>
       <x:c r="M15" s="1"/>
@@ -69943,7 +69948,7 @@
       <x:c r="I16" s="1"/>
       <x:c r="J16" s="1"/>
       <x:c r="K16" s="1" t="str">
-        <x:v>พนักงานบริหารงานทั่วไป</x:v>
+        <x:v>อาจารย์</x:v>
       </x:c>
       <x:c r="L16" s="1"/>
       <x:c r="M16" s="1"/>

</xml_diff>